<commit_message>
Began conversion from v1 WaTCHdb to v2.
</commit_message>
<xml_diff>
--- a/patchr/resources/PLATES_v2.0.0/AB[BATCH_ID].2MPOX.xlsx
+++ b/patchr/resources/PLATES_v2.0.0/AB[BATCH_ID].2MPOX.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/analysis/resources/PLATES_v2.0.0/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/PLATES_v2.0.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B355E0CD-ACD6-284F-8BE5-98BD5E1BE012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E279EBE8-B558-9045-B440-AC1E90155024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="201">
   <si>
     <t>Assay</t>
   </si>
@@ -394,19 +394,10 @@
     <t>Method Lot ID</t>
   </si>
   <si>
-    <t>Target Category</t>
-  </si>
-  <si>
     <t>Target Genetic Locus</t>
   </si>
   <si>
     <t>TD</t>
-  </si>
-  <si>
-    <t>Control 1 Calculated Copies Per uL Reaction</t>
-  </si>
-  <si>
-    <t>Control 2 Calculated Copies Per uL Reaction</t>
   </si>
   <si>
     <t>Input uL</t>
@@ -419,9 +410,6 @@
   </si>
   <si>
     <t>Control 2 Well</t>
-  </si>
-  <si>
-    <t>Target Calculated Copies Per uL Reaction</t>
   </si>
   <si>
     <t>Batch Type</t>
@@ -452,9 +440,6 @@
   </si>
   <si>
     <t>2.0</t>
-  </si>
-  <si>
-    <t>QX Manager Version</t>
   </si>
   <si>
     <t>Zoo QX200</t>
@@ -643,13 +628,22 @@
     <t>Multiple</t>
   </si>
   <si>
-    <t>Target Host</t>
-  </si>
-  <si>
     <t>Mpox Virus Clade I (MPXV)</t>
   </si>
   <si>
     <t>Mpox Virus Clade II (MPXV)</t>
+  </si>
+  <si>
+    <t>Control 1 Predicted Copies Per uL Reaction</t>
+  </si>
+  <si>
+    <t>Control 2 Predicted Copies Per uL Reaction</t>
+  </si>
+  <si>
+    <t>Target Predicted Copies Per uL Reaction</t>
+  </si>
+  <si>
+    <t>Analysis Software Version</t>
   </si>
 </sst>
 </file>
@@ -1377,6 +1371,7 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1408,7 +1403,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1624,7 +1618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D39BBE7-67FA-5442-B147-F43387474561}">
-  <dimension ref="A1:Z910"/>
+  <dimension ref="A1:Z906"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.5703125" style="43" customWidth="1"/>
@@ -1636,7 +1630,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="39" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B1" s="40" t="s">
         <v>0</v>
@@ -1668,7 +1662,7 @@
     </row>
     <row r="2" spans="1:26" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B2" s="45" t="s">
         <v>80</v>
@@ -1735,7 +1729,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C4" s="48"/>
       <c r="D4" s="42"/>
@@ -1767,7 +1761,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="46" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C5" s="42"/>
       <c r="D5" s="42"/>
@@ -1796,10 +1790,10 @@
     </row>
     <row r="6" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="42" t="s">
-        <v>137</v>
+        <v>200</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C6" s="42"/>
       <c r="D6" s="42"/>
@@ -1828,10 +1822,10 @@
     </row>
     <row r="7" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="68" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B7" s="68" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C7" s="42"/>
       <c r="D7" s="42"/>
@@ -1860,13 +1854,13 @@
     </row>
     <row r="8" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="42" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B8" s="42">
         <v>5</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D8" s="42"/>
       <c r="E8" s="42"/>
@@ -1894,7 +1888,7 @@
     </row>
     <row r="9" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="46" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B9" s="46">
         <v>20</v>
@@ -1961,7 +1955,7 @@
         <v>84</v>
       </c>
       <c r="B11" s="46" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C11" s="49"/>
       <c r="D11" s="42"/>
@@ -2022,7 +2016,7 @@
     </row>
     <row r="13" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="46" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B13" s="46" t="s">
         <v>102</v>
@@ -2057,7 +2051,7 @@
         <v>115</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C14" s="49"/>
       <c r="D14" s="42"/>
@@ -2089,7 +2083,7 @@
         <v>116</v>
       </c>
       <c r="B15" s="69" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C15" s="64"/>
       <c r="D15" s="42"/>
@@ -2118,7 +2112,7 @@
     </row>
     <row r="16" spans="1:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="66" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B16" s="67" t="s">
         <v>56</v>
@@ -2150,7 +2144,7 @@
     </row>
     <row r="17" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="65" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B17" s="65" t="s">
         <v>58</v>
@@ -2184,7 +2178,7 @@
         <v>104</v>
       </c>
       <c r="B18" s="50" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C18"/>
       <c r="D18" s="42"/>
@@ -2212,52 +2206,52 @@
       <c r="Z18" s="42"/>
     </row>
     <row r="19" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="50" t="s">
-        <v>200</v>
+      <c r="A19" s="51" t="s">
+        <v>117</v>
       </c>
-      <c r="B19" s="50" t="s">
-        <v>196</v>
+      <c r="B19" s="52" t="s">
+        <v>162</v>
       </c>
       <c r="C19"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="42"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="42"/>
-      <c r="L19" s="42"/>
-      <c r="M19" s="42"/>
-      <c r="N19" s="42"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
-      <c r="T19" s="42"/>
-      <c r="U19" s="42"/>
-      <c r="V19" s="42"/>
-      <c r="W19" s="42"/>
-      <c r="X19" s="42"/>
-      <c r="Y19" s="42"/>
-      <c r="Z19" s="42"/>
     </row>
     <row r="20" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="51" t="s">
-        <v>118</v>
+      <c r="A20" s="50" t="s">
+        <v>78</v>
       </c>
-      <c r="B20" s="52" t="s">
-        <v>167</v>
+      <c r="B20" s="50" t="s">
+        <v>74</v>
       </c>
       <c r="C20"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="42"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="42"/>
+      <c r="O20" s="42"/>
+      <c r="P20" s="42"/>
+      <c r="Q20" s="42"/>
+      <c r="R20" s="42"/>
+      <c r="S20" s="42"/>
+      <c r="T20" s="42"/>
+      <c r="U20" s="42"/>
+      <c r="V20" s="42"/>
+      <c r="W20" s="42"/>
+      <c r="X20" s="42"/>
+      <c r="Y20" s="42"/>
+      <c r="Z20" s="42"/>
     </row>
     <row r="21" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="50" t="s">
-        <v>117</v>
+        <v>199</v>
       </c>
-      <c r="B21" s="50" t="s">
-        <v>98</v>
+      <c r="B21" s="50">
+        <v>0</v>
       </c>
       <c r="C21"/>
       <c r="D21" s="42"/>
@@ -2285,46 +2279,22 @@
       <c r="Z21" s="42"/>
     </row>
     <row r="22" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="50" t="s">
-        <v>78</v>
+      <c r="A22" s="53" t="s">
+        <v>81</v>
       </c>
-      <c r="B22" s="50" t="s">
-        <v>74</v>
+      <c r="B22" s="54" t="s">
+        <v>91</v>
       </c>
       <c r="C22"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="42"/>
-      <c r="K22" s="42"/>
-      <c r="L22" s="42"/>
-      <c r="M22" s="42"/>
-      <c r="N22" s="42"/>
-      <c r="O22" s="42"/>
-      <c r="P22" s="42"/>
-      <c r="Q22" s="42"/>
-      <c r="R22" s="42"/>
-      <c r="S22" s="42"/>
-      <c r="T22" s="42"/>
-      <c r="U22" s="42"/>
-      <c r="V22" s="42"/>
-      <c r="W22" s="42"/>
-      <c r="X22" s="42"/>
-      <c r="Y22" s="42"/>
-      <c r="Z22" s="42"/>
     </row>
     <row r="23" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="50" t="s">
-        <v>126</v>
+      <c r="A23" s="53" t="s">
+        <v>92</v>
       </c>
-      <c r="B23" s="50">
-        <v>0</v>
+      <c r="B23" s="55" t="s">
+        <v>135</v>
       </c>
       <c r="C23"/>
-      <c r="D23" s="42"/>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
       <c r="G23" s="42"/>
@@ -2350,19 +2320,19 @@
     </row>
     <row r="24" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="53" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B24" s="54" t="s">
-        <v>91</v>
+        <v>135</v>
       </c>
       <c r="C24"/>
     </row>
     <row r="25" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="53" t="s">
-        <v>92</v>
+      <c r="A25" s="56" t="s">
+        <v>121</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C25"/>
       <c r="E25" s="42"/>
@@ -2389,22 +2359,45 @@
       <c r="Z25" s="42"/>
     </row>
     <row r="26" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="53" t="s">
-        <v>76</v>
+      <c r="A26" s="56" t="s">
+        <v>197</v>
       </c>
-      <c r="B26" s="54" t="s">
-        <v>140</v>
+      <c r="B26" s="56">
+        <v>0</v>
       </c>
       <c r="C26"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="42"/>
+      <c r="J26" s="42"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="42"/>
+      <c r="N26" s="42"/>
+      <c r="O26" s="42"/>
+      <c r="P26" s="42"/>
+      <c r="Q26" s="42"/>
+      <c r="R26" s="42"/>
+      <c r="S26" s="42"/>
+      <c r="T26" s="42"/>
+      <c r="U26" s="42"/>
+      <c r="V26" s="42"/>
+      <c r="W26" s="42"/>
+      <c r="X26" s="42"/>
+      <c r="Y26" s="42"/>
+      <c r="Z26" s="42"/>
     </row>
     <row r="27" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="56" t="s">
-        <v>124</v>
+      <c r="A27" s="57" t="s">
+        <v>82</v>
       </c>
-      <c r="B27" s="55" t="s">
-        <v>146</v>
+      <c r="B27" s="58" t="s">
+        <v>90</v>
       </c>
       <c r="C27"/>
+      <c r="D27" s="42"/>
       <c r="E27" s="42"/>
       <c r="F27" s="42"/>
       <c r="G27" s="42"/>
@@ -2429,13 +2422,14 @@
       <c r="Z27" s="42"/>
     </row>
     <row r="28" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="56" t="s">
-        <v>120</v>
+      <c r="A28" s="59" t="s">
+        <v>93</v>
       </c>
-      <c r="B28" s="56">
-        <v>0</v>
+      <c r="B28" s="59" t="s">
+        <v>96</v>
       </c>
       <c r="C28"/>
+      <c r="D28" s="42"/>
       <c r="E28" s="42"/>
       <c r="F28" s="42"/>
       <c r="G28" s="42"/>
@@ -2461,10 +2455,10 @@
     </row>
     <row r="29" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="57" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
-      <c r="B29" s="58" t="s">
-        <v>90</v>
+      <c r="B29" s="60" t="s">
+        <v>74</v>
       </c>
       <c r="C29"/>
       <c r="D29" s="42"/>
@@ -2493,10 +2487,10 @@
     </row>
     <row r="30" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="59" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="B30" s="59" t="s">
-        <v>96</v>
+        <v>141</v>
       </c>
       <c r="C30"/>
       <c r="D30" s="42"/>
@@ -2523,14 +2517,14 @@
       <c r="Y30" s="42"/>
       <c r="Z30" s="42"/>
     </row>
-    <row r="31" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="57" t="s">
-        <v>77</v>
+    <row r="31" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="62" t="s">
+        <v>198</v>
       </c>
-      <c r="B31" s="60" t="s">
-        <v>74</v>
+      <c r="B31" s="59">
+        <v>100</v>
       </c>
-      <c r="C31"/>
+      <c r="C31" s="74"/>
       <c r="D31" s="42"/>
       <c r="E31" s="42"/>
       <c r="F31" s="42"/>
@@ -2555,12 +2549,12 @@
       <c r="Y31" s="42"/>
       <c r="Z31" s="42"/>
     </row>
-    <row r="32" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="59" t="s">
-        <v>125</v>
+    <row r="32" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="65" t="s">
+        <v>127</v>
       </c>
-      <c r="B32" s="59" t="s">
-        <v>146</v>
+      <c r="B32" s="61" t="s">
+        <v>60</v>
       </c>
       <c r="C32"/>
       <c r="D32" s="42"/>
@@ -2587,14 +2581,14 @@
       <c r="Y32" s="42"/>
       <c r="Z32" s="42"/>
     </row>
-    <row r="33" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="62" t="s">
-        <v>121</v>
+    <row r="33" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="50" t="s">
+        <v>104</v>
       </c>
-      <c r="B33" s="59">
-        <v>100</v>
+      <c r="B33" s="50" t="s">
+        <v>196</v>
       </c>
-      <c r="C33" s="89"/>
+      <c r="C33"/>
       <c r="D33" s="42"/>
       <c r="E33" s="42"/>
       <c r="F33" s="42"/>
@@ -2620,11 +2614,11 @@
       <c r="Z33" s="42"/>
     </row>
     <row r="34" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="65" t="s">
-        <v>131</v>
+      <c r="A34" s="51" t="s">
+        <v>117</v>
       </c>
-      <c r="B34" s="61" t="s">
-        <v>60</v>
+      <c r="B34" s="52" t="s">
+        <v>161</v>
       </c>
       <c r="C34"/>
       <c r="D34" s="42"/>
@@ -2653,10 +2647,10 @@
     </row>
     <row r="35" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="50" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="B35" s="50" t="s">
-        <v>202</v>
+        <v>74</v>
       </c>
       <c r="C35"/>
       <c r="D35" s="42"/>
@@ -2683,12 +2677,12 @@
       <c r="Y35" s="42"/>
       <c r="Z35" s="42"/>
     </row>
-    <row r="36" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="50" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
-      <c r="B36" s="50" t="s">
-        <v>196</v>
+      <c r="B36" s="50">
+        <v>0</v>
       </c>
       <c r="C36"/>
       <c r="D36" s="42"/>
@@ -2716,11 +2710,11 @@
       <c r="Z36" s="42"/>
     </row>
     <row r="37" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="51" t="s">
-        <v>118</v>
+      <c r="A37" s="53" t="s">
+        <v>81</v>
       </c>
-      <c r="B37" s="52" t="s">
-        <v>166</v>
+      <c r="B37" s="54" t="s">
+        <v>91</v>
       </c>
       <c r="C37"/>
       <c r="D37" s="42"/>
@@ -2748,11 +2742,11 @@
       <c r="Z37" s="42"/>
     </row>
     <row r="38" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="50" t="s">
-        <v>117</v>
+      <c r="A38" s="53" t="s">
+        <v>92</v>
       </c>
-      <c r="B38" s="50" t="s">
-        <v>98</v>
+      <c r="B38" s="55" t="s">
+        <v>135</v>
       </c>
       <c r="C38"/>
       <c r="D38" s="42"/>
@@ -2780,11 +2774,11 @@
       <c r="Z38" s="42"/>
     </row>
     <row r="39" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="50" t="s">
-        <v>78</v>
+      <c r="A39" s="53" t="s">
+        <v>76</v>
       </c>
-      <c r="B39" s="50" t="s">
-        <v>74</v>
+      <c r="B39" s="54" t="s">
+        <v>135</v>
       </c>
       <c r="C39"/>
       <c r="D39" s="42"/>
@@ -2812,11 +2806,11 @@
       <c r="Z39" s="42"/>
     </row>
     <row r="40" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="50" t="s">
-        <v>126</v>
+      <c r="A40" s="56" t="s">
+        <v>121</v>
       </c>
-      <c r="B40" s="50">
-        <v>0</v>
+      <c r="B40" s="55" t="s">
+        <v>141</v>
       </c>
       <c r="C40"/>
       <c r="D40" s="42"/>
@@ -2844,11 +2838,11 @@
       <c r="Z40" s="42"/>
     </row>
     <row r="41" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="53" t="s">
-        <v>81</v>
+      <c r="A41" s="56" t="s">
+        <v>197</v>
       </c>
-      <c r="B41" s="54" t="s">
-        <v>91</v>
+      <c r="B41" s="56">
+        <v>0</v>
       </c>
       <c r="C41"/>
       <c r="D41" s="42"/>
@@ -2876,11 +2870,11 @@
       <c r="Z41" s="42"/>
     </row>
     <row r="42" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="53" t="s">
-        <v>92</v>
+      <c r="A42" s="57" t="s">
+        <v>82</v>
       </c>
-      <c r="B42" s="55" t="s">
-        <v>140</v>
+      <c r="B42" s="58" t="s">
+        <v>90</v>
       </c>
       <c r="C42"/>
       <c r="D42" s="42"/>
@@ -2908,11 +2902,11 @@
       <c r="Z42" s="42"/>
     </row>
     <row r="43" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="53" t="s">
-        <v>76</v>
+      <c r="A43" s="59" t="s">
+        <v>93</v>
       </c>
-      <c r="B43" s="54" t="s">
-        <v>140</v>
+      <c r="B43" s="59" t="s">
+        <v>96</v>
       </c>
       <c r="C43"/>
       <c r="D43" s="42"/>
@@ -2940,11 +2934,11 @@
       <c r="Z43" s="42"/>
     </row>
     <row r="44" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="56" t="s">
-        <v>124</v>
+      <c r="A44" s="57" t="s">
+        <v>77</v>
       </c>
-      <c r="B44" s="55" t="s">
-        <v>146</v>
+      <c r="B44" s="60" t="s">
+        <v>74</v>
       </c>
       <c r="C44"/>
       <c r="D44" s="42"/>
@@ -2972,11 +2966,11 @@
       <c r="Z44" s="42"/>
     </row>
     <row r="45" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="56" t="s">
-        <v>120</v>
+      <c r="A45" s="59" t="s">
+        <v>122</v>
       </c>
-      <c r="B45" s="56">
-        <v>0</v>
+      <c r="B45" s="59" t="s">
+        <v>141</v>
       </c>
       <c r="C45"/>
       <c r="D45" s="42"/>
@@ -3003,14 +2997,14 @@
       <c r="Y45" s="42"/>
       <c r="Z45" s="42"/>
     </row>
-    <row r="46" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="57" t="s">
-        <v>82</v>
+    <row r="46" spans="1:26" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="62" t="s">
+        <v>198</v>
       </c>
-      <c r="B46" s="58" t="s">
-        <v>90</v>
+      <c r="B46" s="62">
+        <v>100</v>
       </c>
-      <c r="C46"/>
+      <c r="C46" s="74"/>
       <c r="D46" s="42"/>
       <c r="E46" s="42"/>
       <c r="F46" s="42"/>
@@ -3035,138 +3029,122 @@
       <c r="Y46" s="42"/>
       <c r="Z46" s="42"/>
     </row>
-    <row r="47" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="59" t="s">
-        <v>93</v>
-      </c>
-      <c r="B47" s="59" t="s">
-        <v>96</v>
-      </c>
-      <c r="C47"/>
-      <c r="D47" s="42"/>
-      <c r="E47" s="42"/>
-      <c r="F47" s="42"/>
-      <c r="G47" s="42"/>
-      <c r="H47" s="42"/>
-      <c r="I47" s="42"/>
-      <c r="J47" s="42"/>
-      <c r="K47" s="42"/>
-      <c r="L47" s="42"/>
-      <c r="M47" s="42"/>
-      <c r="N47" s="42"/>
-      <c r="O47" s="42"/>
-      <c r="P47" s="42"/>
-      <c r="Q47" s="42"/>
-      <c r="R47" s="42"/>
-      <c r="S47" s="42"/>
-      <c r="T47" s="42"/>
-      <c r="U47" s="42"/>
-      <c r="V47" s="42"/>
-      <c r="W47" s="42"/>
-      <c r="X47" s="42"/>
-      <c r="Y47" s="42"/>
-      <c r="Z47" s="42"/>
-    </row>
-    <row r="48" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="57" t="s">
-        <v>77</v>
-      </c>
-      <c r="B48" s="60" t="s">
-        <v>74</v>
-      </c>
-      <c r="C48"/>
-      <c r="D48" s="42"/>
-      <c r="E48" s="42"/>
-      <c r="F48" s="42"/>
-      <c r="G48" s="42"/>
-      <c r="H48" s="42"/>
-      <c r="I48" s="42"/>
-      <c r="J48" s="42"/>
-      <c r="K48" s="42"/>
-      <c r="L48" s="42"/>
-      <c r="M48" s="42"/>
-      <c r="N48" s="42"/>
-      <c r="O48" s="42"/>
-      <c r="P48" s="42"/>
-      <c r="Q48" s="42"/>
-      <c r="R48" s="42"/>
-      <c r="S48" s="42"/>
-      <c r="T48" s="42"/>
-      <c r="U48" s="42"/>
-      <c r="V48" s="42"/>
-      <c r="W48" s="42"/>
-      <c r="X48" s="42"/>
-      <c r="Y48" s="42"/>
-      <c r="Z48" s="42"/>
-    </row>
-    <row r="49" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="59" t="s">
-        <v>125</v>
-      </c>
-      <c r="B49" s="59" t="s">
-        <v>146</v>
-      </c>
-      <c r="C49"/>
-      <c r="D49" s="42"/>
-      <c r="E49" s="42"/>
-      <c r="F49" s="42"/>
-      <c r="G49" s="42"/>
-      <c r="H49" s="42"/>
-      <c r="I49" s="42"/>
-      <c r="J49" s="42"/>
-      <c r="K49" s="42"/>
-      <c r="L49" s="42"/>
-      <c r="M49" s="42"/>
-      <c r="N49" s="42"/>
-      <c r="O49" s="42"/>
-      <c r="P49" s="42"/>
-      <c r="Q49" s="42"/>
-      <c r="R49" s="42"/>
-      <c r="S49" s="42"/>
-      <c r="T49" s="42"/>
-      <c r="U49" s="42"/>
-      <c r="V49" s="42"/>
-      <c r="W49" s="42"/>
-      <c r="X49" s="42"/>
-      <c r="Y49" s="42"/>
-      <c r="Z49" s="42"/>
-    </row>
-    <row r="50" spans="1:26" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="62" t="s">
-        <v>121</v>
-      </c>
-      <c r="B50" s="62">
-        <v>100</v>
-      </c>
-      <c r="C50" s="89"/>
-      <c r="D50" s="42"/>
-      <c r="E50" s="42"/>
-      <c r="F50" s="42"/>
-      <c r="G50" s="42"/>
-      <c r="H50" s="42"/>
-      <c r="I50" s="42"/>
-      <c r="J50" s="42"/>
-      <c r="K50" s="42"/>
-      <c r="L50" s="42"/>
-      <c r="M50" s="42"/>
-      <c r="N50" s="42"/>
-      <c r="O50" s="42"/>
-      <c r="P50" s="42"/>
-      <c r="Q50" s="42"/>
-      <c r="R50" s="42"/>
-      <c r="S50" s="42"/>
-      <c r="T50" s="42"/>
-      <c r="U50" s="42"/>
-      <c r="V50" s="42"/>
-      <c r="W50" s="42"/>
-      <c r="X50" s="42"/>
-      <c r="Y50" s="42"/>
-      <c r="Z50" s="42"/>
-    </row>
-    <row r="51" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="52" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="53" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="54" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="49" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="50" spans="1:26" s="63" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="51" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="42"/>
+      <c r="B51" s="42"/>
+      <c r="C51" s="42"/>
+      <c r="D51" s="42"/>
+      <c r="E51" s="42"/>
+      <c r="F51" s="42"/>
+      <c r="G51" s="42"/>
+      <c r="H51" s="42"/>
+      <c r="I51" s="42"/>
+      <c r="J51" s="42"/>
+      <c r="K51" s="42"/>
+      <c r="L51" s="42"/>
+      <c r="M51" s="42"/>
+      <c r="N51" s="42"/>
+      <c r="O51" s="42"/>
+      <c r="P51" s="42"/>
+      <c r="Q51" s="42"/>
+      <c r="R51" s="42"/>
+      <c r="S51" s="42"/>
+      <c r="T51" s="42"/>
+      <c r="U51" s="42"/>
+      <c r="V51" s="42"/>
+      <c r="W51" s="42"/>
+      <c r="X51" s="42"/>
+      <c r="Y51" s="42"/>
+      <c r="Z51" s="42"/>
+    </row>
+    <row r="52" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="42"/>
+      <c r="B52" s="42"/>
+      <c r="C52" s="42"/>
+      <c r="D52" s="42"/>
+      <c r="E52" s="42"/>
+      <c r="F52" s="42"/>
+      <c r="G52" s="42"/>
+      <c r="H52" s="42"/>
+      <c r="I52" s="42"/>
+      <c r="J52" s="42"/>
+      <c r="K52" s="42"/>
+      <c r="L52" s="42"/>
+      <c r="M52" s="42"/>
+      <c r="N52" s="42"/>
+      <c r="O52" s="42"/>
+      <c r="P52" s="42"/>
+      <c r="Q52" s="42"/>
+      <c r="R52" s="42"/>
+      <c r="S52" s="42"/>
+      <c r="T52" s="42"/>
+      <c r="U52" s="42"/>
+      <c r="V52" s="42"/>
+      <c r="W52" s="42"/>
+      <c r="X52" s="42"/>
+      <c r="Y52" s="42"/>
+      <c r="Z52" s="42"/>
+    </row>
+    <row r="53" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="42"/>
+      <c r="B53" s="42"/>
+      <c r="C53" s="42"/>
+      <c r="D53" s="42"/>
+      <c r="E53" s="42"/>
+      <c r="F53" s="42"/>
+      <c r="G53" s="42"/>
+      <c r="H53" s="42"/>
+      <c r="I53" s="42"/>
+      <c r="J53" s="42"/>
+      <c r="K53" s="42"/>
+      <c r="L53" s="42"/>
+      <c r="M53" s="42"/>
+      <c r="N53" s="42"/>
+      <c r="O53" s="42"/>
+      <c r="P53" s="42"/>
+      <c r="Q53" s="42"/>
+      <c r="R53" s="42"/>
+      <c r="S53" s="42"/>
+      <c r="T53" s="42"/>
+      <c r="U53" s="42"/>
+      <c r="V53" s="42"/>
+      <c r="W53" s="42"/>
+      <c r="X53" s="42"/>
+      <c r="Y53" s="42"/>
+      <c r="Z53" s="42"/>
+    </row>
+    <row r="54" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="42"/>
+      <c r="B54" s="42"/>
+      <c r="C54" s="42"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="42"/>
+      <c r="F54" s="42"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="42"/>
+      <c r="I54" s="42"/>
+      <c r="J54" s="42"/>
+      <c r="K54" s="42"/>
+      <c r="L54" s="42"/>
+      <c r="M54" s="42"/>
+      <c r="N54" s="42"/>
+      <c r="O54" s="42"/>
+      <c r="P54" s="42"/>
+      <c r="Q54" s="42"/>
+      <c r="R54" s="42"/>
+      <c r="S54" s="42"/>
+      <c r="T54" s="42"/>
+      <c r="U54" s="42"/>
+      <c r="V54" s="42"/>
+      <c r="W54" s="42"/>
+      <c r="X54" s="42"/>
+      <c r="Y54" s="42"/>
+      <c r="Z54" s="42"/>
+    </row>
     <row r="55" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="42"/>
       <c r="B55" s="42"/>
@@ -27023,129 +27001,17 @@
       <c r="Y906" s="42"/>
       <c r="Z906" s="42"/>
     </row>
-    <row r="907" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A907" s="42"/>
-      <c r="B907" s="42"/>
-      <c r="C907" s="42"/>
-      <c r="D907" s="42"/>
-      <c r="E907" s="42"/>
-      <c r="F907" s="42"/>
-      <c r="G907" s="42"/>
-      <c r="H907" s="42"/>
-      <c r="I907" s="42"/>
-      <c r="J907" s="42"/>
-      <c r="K907" s="42"/>
-      <c r="L907" s="42"/>
-      <c r="M907" s="42"/>
-      <c r="N907" s="42"/>
-      <c r="O907" s="42"/>
-      <c r="P907" s="42"/>
-      <c r="Q907" s="42"/>
-      <c r="R907" s="42"/>
-      <c r="S907" s="42"/>
-      <c r="T907" s="42"/>
-      <c r="U907" s="42"/>
-      <c r="V907" s="42"/>
-      <c r="W907" s="42"/>
-      <c r="X907" s="42"/>
-      <c r="Y907" s="42"/>
-      <c r="Z907" s="42"/>
-    </row>
-    <row r="908" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A908" s="42"/>
-      <c r="B908" s="42"/>
-      <c r="C908" s="42"/>
-      <c r="D908" s="42"/>
-      <c r="E908" s="42"/>
-      <c r="F908" s="42"/>
-      <c r="G908" s="42"/>
-      <c r="H908" s="42"/>
-      <c r="I908" s="42"/>
-      <c r="J908" s="42"/>
-      <c r="K908" s="42"/>
-      <c r="L908" s="42"/>
-      <c r="M908" s="42"/>
-      <c r="N908" s="42"/>
-      <c r="O908" s="42"/>
-      <c r="P908" s="42"/>
-      <c r="Q908" s="42"/>
-      <c r="R908" s="42"/>
-      <c r="S908" s="42"/>
-      <c r="T908" s="42"/>
-      <c r="U908" s="42"/>
-      <c r="V908" s="42"/>
-      <c r="W908" s="42"/>
-      <c r="X908" s="42"/>
-      <c r="Y908" s="42"/>
-      <c r="Z908" s="42"/>
-    </row>
-    <row r="909" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A909" s="42"/>
-      <c r="B909" s="42"/>
-      <c r="C909" s="42"/>
-      <c r="D909" s="42"/>
-      <c r="E909" s="42"/>
-      <c r="F909" s="42"/>
-      <c r="G909" s="42"/>
-      <c r="H909" s="42"/>
-      <c r="I909" s="42"/>
-      <c r="J909" s="42"/>
-      <c r="K909" s="42"/>
-      <c r="L909" s="42"/>
-      <c r="M909" s="42"/>
-      <c r="N909" s="42"/>
-      <c r="O909" s="42"/>
-      <c r="P909" s="42"/>
-      <c r="Q909" s="42"/>
-      <c r="R909" s="42"/>
-      <c r="S909" s="42"/>
-      <c r="T909" s="42"/>
-      <c r="U909" s="42"/>
-      <c r="V909" s="42"/>
-      <c r="W909" s="42"/>
-      <c r="X909" s="42"/>
-      <c r="Y909" s="42"/>
-      <c r="Z909" s="42"/>
-    </row>
-    <row r="910" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A910" s="42"/>
-      <c r="B910" s="42"/>
-      <c r="C910" s="42"/>
-      <c r="D910" s="42"/>
-      <c r="E910" s="42"/>
-      <c r="F910" s="42"/>
-      <c r="G910" s="42"/>
-      <c r="H910" s="42"/>
-      <c r="I910" s="42"/>
-      <c r="J910" s="42"/>
-      <c r="K910" s="42"/>
-      <c r="L910" s="42"/>
-      <c r="M910" s="42"/>
-      <c r="N910" s="42"/>
-      <c r="O910" s="42"/>
-      <c r="P910" s="42"/>
-      <c r="Q910" s="42"/>
-      <c r="R910" s="42"/>
-      <c r="S910" s="42"/>
-      <c r="T910" s="42"/>
-      <c r="U910" s="42"/>
-      <c r="V910" s="42"/>
-      <c r="W910" s="42"/>
-      <c r="X910" s="42"/>
-      <c r="Y910" s="42"/>
-      <c r="Z910" s="42"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="20">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="16">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9269EC84-DF31-1A4B-A990-FD99E0DF6A37}">
           <x14:formula1>
             <xm:f>Lists!$F$2:$F$10</xm:f>
           </x14:formula1>
-          <xm:sqref>B30 B25 B47 B42</xm:sqref>
+          <xm:sqref>B28 B23 B43 B38</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F48AC468-AC67-414F-A31D-152D1C1A14B8}">
           <x14:formula1>
@@ -27157,7 +27023,7 @@
           <x14:formula1>
             <xm:f>Lists!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B41 B46 B24 B29</xm:sqref>
+          <xm:sqref>B37 B42 B22 B27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{FFB11884-705E-4C4B-9963-11B4FBF86EFD}">
           <x14:formula1>
@@ -27181,7 +27047,7 @@
           <x14:formula1>
             <xm:f>Lists!$E$2:$E$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B26 B31 B43 B48 B22 B39</xm:sqref>
+          <xm:sqref>B24 B29 B39 B44 B20 B35</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{8B68413C-BA2E-3E4F-BCCD-63E54D16131E}">
           <x14:formula1>
@@ -27193,31 +27059,19 @@
           <x14:formula1>
             <xm:f>Lists!$G$3:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B41</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{C159AD43-387F-8A44-88E8-16412071B24C}">
-          <x14:formula1>
-            <xm:f>Lists!$C$2:$C$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>B21 B38</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FF158337-349C-AE45-9DC7-81D1DD942C51}">
-          <x14:formula1>
-            <xm:f>Lists!$C$2:$C$9</xm:f>
-          </x14:formula1>
-          <xm:sqref>B38 B21</xm:sqref>
+          <xm:sqref>B37</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8F92160A-7435-3B42-84F3-7B849CE421F0}">
           <x14:formula1>
             <xm:f>Lists!$H$2:$H$7</xm:f>
           </x14:formula1>
-          <xm:sqref>B34 B17</xm:sqref>
+          <xm:sqref>B32 B17</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{209ABDC6-7A4F-1043-BD31-F5067EDD9592}">
           <x14:formula1>
             <xm:f>Lists!$D$2:$D$27</xm:f>
           </x14:formula1>
-          <xm:sqref>B37 B20</xm:sqref>
+          <xm:sqref>B34 B19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{4DE4111E-DA5E-784E-9D6F-05103F7D2493}">
           <x14:formula1>
@@ -27225,35 +27079,23 @@
           </x14:formula1>
           <xm:sqref>B14</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{458F1957-7F4C-3843-8AFA-688CEDE96E83}">
-          <x14:formula1>
-            <xm:f>Lists!$N$2:$N$7</xm:f>
-          </x14:formula1>
-          <xm:sqref>B19 B36</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B241593E-F5D9-0643-9841-833D07C14BE8}">
-          <x14:formula1>
-            <xm:f>Lists!$N$2:$N$7</xm:f>
-          </x14:formula1>
-          <xm:sqref>B19 B36</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{970994F8-0C5A-954C-8A5B-082DB9E55E96}">
           <x14:formula1>
             <xm:f>Lists!$B$2:$B$27</xm:f>
           </x14:formula1>
-          <xm:sqref>B35 B18</xm:sqref>
+          <xm:sqref>B33 B18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F9DEF641-EE3D-B047-8D16-CAC81DB4BCBD}">
           <x14:formula1>
             <xm:f>Lists!$B$2:$B$17</xm:f>
           </x14:formula1>
-          <xm:sqref>B35</xm:sqref>
+          <xm:sqref>B33</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C377399E-4DEA-7E44-B16E-7301589BBC04}">
           <x14:formula1>
             <xm:f>Lists!$B$3:$B$27</xm:f>
           </x14:formula1>
-          <xm:sqref>B35</xm:sqref>
+          <xm:sqref>B33</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4B8BFAEF-3C0C-4641-836E-A751B7E93527}">
           <x14:formula1>
@@ -39991,40 +39833,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="81" t="s">
+      <c r="A1" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="82"/>
-      <c r="M1" s="82"/>
-      <c r="N1" s="82"/>
-      <c r="O1" s="82"/>
-      <c r="P1" s="82"/>
-      <c r="Q1" s="83"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="83"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="84"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
     </row>
     <row r="2" spans="1:19" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="88" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="87"/>
-      <c r="I2" s="87"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -40035,17 +39877,17 @@
       <c r="S2" s="2"/>
     </row>
     <row r="3" spans="1:19" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="88" t="s">
+      <c r="A3" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -40102,11 +39944,11 @@
       <c r="B6" s="10">
         <v>16.5</v>
       </c>
-      <c r="C6" s="77" t="s">
+      <c r="C6" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="78"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
@@ -40122,9 +39964,9 @@
       <c r="B7" s="10">
         <v>5.5</v>
       </c>
-      <c r="C7" s="78"/>
-      <c r="D7" s="78"/>
-      <c r="E7" s="78"/>
+      <c r="C7" s="79"/>
+      <c r="D7" s="79"/>
+      <c r="E7" s="79"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
@@ -40141,9 +39983,9 @@
         <f>SUM(B6:B7)</f>
         <v>22</v>
       </c>
-      <c r="C8" s="78"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="78"/>
+      <c r="C8" s="79"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="79"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
@@ -40159,9 +40001,9 @@
       <c r="B9" s="10">
         <v>20</v>
       </c>
-      <c r="C9" s="78"/>
-      <c r="D9" s="78"/>
-      <c r="E9" s="78"/>
+      <c r="C9" s="79"/>
+      <c r="D9" s="79"/>
+      <c r="E9" s="79"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
@@ -40185,12 +40027,12 @@
       <c r="L10" s="8"/>
     </row>
     <row r="11" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="84" t="s">
+      <c r="A11" s="85" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="82"/>
-      <c r="C11" s="82"/>
-      <c r="D11" s="83"/>
+      <c r="B11" s="83"/>
+      <c r="C11" s="83"/>
+      <c r="D11" s="84"/>
       <c r="E11" s="12"/>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
@@ -40254,7 +40096,7 @@
       <c r="C15" s="17">
         <v>0.5</v>
       </c>
-      <c r="D15" s="85">
+      <c r="D15" s="86">
         <v>40</v>
       </c>
     </row>
@@ -40268,7 +40110,7 @@
       <c r="C16" s="17">
         <v>1</v>
       </c>
-      <c r="D16" s="86"/>
+      <c r="D16" s="87"/>
     </row>
     <row r="17" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
@@ -40291,12 +40133,12 @@
       <c r="D18" s="12"/>
     </row>
     <row r="19" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="74" t="s">
+      <c r="A19" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="75"/>
-      <c r="C19" s="75"/>
-      <c r="D19" s="76"/>
+      <c r="B19" s="76"/>
+      <c r="C19" s="76"/>
+      <c r="D19" s="77"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
@@ -40337,18 +40179,18 @@
         <f>COUNTIF('Sample IDs'!B2:M9,"&lt;&gt;"&amp;"")</f>
         <v>0</v>
       </c>
-      <c r="C24" s="77" t="s">
+      <c r="C24" s="78" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="78"/>
-      <c r="E24" s="78"/>
-      <c r="F24" s="78"/>
-      <c r="G24" s="78"/>
-      <c r="H24" s="78"/>
-      <c r="I24" s="78"/>
-      <c r="J24" s="78"/>
-      <c r="K24" s="78"/>
-      <c r="L24" s="78"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="79"/>
+      <c r="F24" s="79"/>
+      <c r="G24" s="79"/>
+      <c r="H24" s="79"/>
+      <c r="I24" s="79"/>
+      <c r="J24" s="79"/>
+      <c r="K24" s="79"/>
+      <c r="L24" s="79"/>
     </row>
     <row r="25" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="23" t="s">
@@ -40385,10 +40227,10 @@
       <c r="L26" s="8"/>
     </row>
     <row r="27" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="79" t="s">
+      <c r="A27" s="80" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="80"/>
+      <c r="B27" s="81"/>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
       <c r="E27" s="12"/>
@@ -41523,10 +41365,10 @@
         <v>105</v>
       </c>
       <c r="D1" s="70" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E1" s="71" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="F1" s="70" t="s">
         <v>94</v>
@@ -41550,33 +41392,33 @@
         <v>55</v>
       </c>
       <c r="M1" s="71" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="N1" s="71" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="63" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B2" s="63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C2" s="63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D2" s="63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E2" s="63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F2" s="63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="G2" s="63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="H2" s="63" t="s">
         <v>58</v>
@@ -41594,24 +41436,24 @@
         <v>70</v>
       </c>
       <c r="M2" s="72" t="s">
+        <v>131</v>
+      </c>
+      <c r="N2" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="N2" s="63" t="s">
-        <v>140</v>
-      </c>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="63" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B3" s="63" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C3" s="63" t="s">
         <v>98</v>
       </c>
       <c r="D3" s="63" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="E3" s="63" t="s">
         <v>74</v>
@@ -41635,13 +41477,13 @@
         <v>61</v>
       </c>
       <c r="L3" s="63" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="M3" s="72" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="N3" s="63" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -41652,10 +41494,10 @@
         <v>101</v>
       </c>
       <c r="C4" s="63" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D4" s="63" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E4" s="63" t="s">
         <v>73</v>
@@ -41679,11 +41521,11 @@
         <v>103</v>
       </c>
       <c r="L4" s="63" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="M4" s="63"/>
       <c r="N4" s="63" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -41695,7 +41537,7 @@
         <v>99</v>
       </c>
       <c r="D5" s="63" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E5" s="63" t="s">
         <v>79</v>
@@ -41715,23 +41557,23 @@
         <v>69</v>
       </c>
       <c r="L5" s="63" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="M5" s="63"/>
       <c r="N5" s="63" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="63"/>
       <c r="B6" s="63" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C6" s="63" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="63" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E6" s="63" t="s">
         <v>69</v>
@@ -41741,23 +41583,23 @@
       </c>
       <c r="G6" s="63"/>
       <c r="H6" s="63" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="I6" s="63"/>
       <c r="J6" s="63"/>
       <c r="K6" s="63"/>
       <c r="L6" s="63" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="M6" s="63"/>
       <c r="N6" s="63" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="63"/>
       <c r="B7" s="73" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C7" s="63"/>
       <c r="D7" s="63" t="s">
@@ -41769,13 +41611,13 @@
       </c>
       <c r="G7" s="63"/>
       <c r="H7" s="63" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="I7" s="63"/>
       <c r="J7" s="63"/>
       <c r="K7" s="63"/>
       <c r="L7" s="63" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="M7" s="63"/>
       <c r="N7" s="63" t="s">
@@ -41785,7 +41627,7 @@
     <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="63"/>
       <c r="B8" s="63" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C8" s="63"/>
       <c r="D8" s="63" t="s">
@@ -41803,14 +41645,14 @@
       <c r="J8" s="63"/>
       <c r="K8" s="63"/>
       <c r="L8" s="63" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M8" s="63"/>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="63"/>
       <c r="B9" s="63" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C9" s="63"/>
       <c r="D9" s="63" t="s">
@@ -41828,18 +41670,18 @@
       <c r="J9" s="63"/>
       <c r="K9" s="63"/>
       <c r="L9" s="63" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="M9" s="63"/>
     </row>
     <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="63"/>
       <c r="B10" s="73" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C10" s="63"/>
       <c r="D10" s="63" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E10" s="63"/>
       <c r="F10" s="63" t="s">
@@ -41851,18 +41693,18 @@
       <c r="J10" s="63"/>
       <c r="K10" s="63"/>
       <c r="L10" s="63" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="M10" s="63"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="63"/>
       <c r="B11" s="73" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C11" s="63"/>
       <c r="D11" s="63" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E11" s="63"/>
       <c r="F11" s="63"/>
@@ -41872,18 +41714,18 @@
       <c r="J11" s="63"/>
       <c r="K11" s="63"/>
       <c r="L11" s="63" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="M11" s="63"/>
     </row>
     <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="63"/>
       <c r="B12" s="63" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C12" s="63"/>
       <c r="D12" s="63" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E12" s="63"/>
       <c r="F12" s="63"/>
@@ -41893,18 +41735,18 @@
       <c r="J12" s="63"/>
       <c r="K12" s="63"/>
       <c r="L12" s="63" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="M12" s="63"/>
     </row>
     <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="63"/>
       <c r="B13" s="63" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C13" s="63"/>
       <c r="D13" s="63" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E13" s="63"/>
       <c r="F13" s="63"/>
@@ -41914,18 +41756,18 @@
       <c r="J13" s="63"/>
       <c r="K13" s="63"/>
       <c r="L13" s="63" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="M13" s="63"/>
     </row>
     <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="63"/>
       <c r="B14" s="63" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C14" s="63"/>
       <c r="D14" s="63" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E14" s="63"/>
       <c r="F14" s="63"/>
@@ -41935,18 +41777,18 @@
       <c r="J14" s="63"/>
       <c r="K14" s="63"/>
       <c r="L14" s="63" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="M14" s="63"/>
     </row>
     <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="63"/>
       <c r="B15" s="63" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C15" s="63"/>
       <c r="D15" s="63" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E15" s="63"/>
       <c r="F15" s="63"/>
@@ -41956,18 +41798,18 @@
       <c r="J15" s="63"/>
       <c r="K15" s="63"/>
       <c r="L15" s="63" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="M15" s="63"/>
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="63"/>
       <c r="B16" s="63" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C16" s="63"/>
       <c r="D16" s="63" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="E16" s="63"/>
       <c r="F16" s="63"/>
@@ -41977,18 +41819,18 @@
       <c r="J16" s="63"/>
       <c r="K16" s="63"/>
       <c r="L16" s="63" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="M16" s="63"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="63"/>
       <c r="B17" s="63" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C17" s="63"/>
       <c r="D17" s="63" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="E17" s="63"/>
       <c r="F17" s="63"/>
@@ -42019,14 +41861,14 @@
       <c r="J18" s="63"/>
       <c r="K18" s="63"/>
       <c r="L18" s="63" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="M18" s="63"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="63"/>
       <c r="B19" s="63" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C19" s="63"/>
       <c r="D19" s="63" t="s">
@@ -42044,7 +41886,7 @@
     <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="63"/>
       <c r="B20" s="63" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C20" s="63"/>
       <c r="D20" s="63" t="s">
@@ -42062,7 +41904,7 @@
     <row r="21" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="63"/>
       <c r="B21" s="73" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C21" s="63"/>
       <c r="D21" s="63" t="s">
@@ -42081,7 +41923,7 @@
     <row r="22" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="63"/>
       <c r="B22" s="73" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C22" s="63"/>
       <c r="D22" s="63" t="s">
@@ -42100,7 +41942,7 @@
     <row r="23" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="63"/>
       <c r="B23" s="73" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C23" s="63"/>
       <c r="D23" s="63" t="s">
@@ -42119,7 +41961,7 @@
     <row r="24" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="63"/>
       <c r="B24" s="73" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C24" s="63"/>
       <c r="D24" s="63" t="s">
@@ -42138,7 +41980,7 @@
     <row r="25" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="63"/>
       <c r="B25" s="73" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C25" s="63"/>
       <c r="D25" s="63" t="s">
@@ -42159,7 +42001,7 @@
         <v>71</v>
       </c>
       <c r="D26" s="63" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>